<commit_message>
Paso 7: Refinamiento UX Voyage Ledger - TBD logic, separadores de miles, fix fecha bunker, compresion layout, fix unidad v_intake, limpieza 9999 en DB
</commit_message>
<xml_diff>
--- a/Exceles.Petral/Naviera Petral -Margen de Operacion 2026 - 11.junio.2026.xlsx
+++ b/Exceles.Petral/Naviera Petral -Margen de Operacion 2026 - 11.junio.2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\MARGEN OPERACIONAL CONSOLIDADO FH\2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rguti\PETRAL.SMART.DASHBOARD\Exceles.Petral\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7119E752-1E31-49DC-AE50-AF499FC9D92A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14C1CF35-AB86-4C6F-BC05-683A01E6CD98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="617" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="617" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONSOLIDADO " sheetId="7" r:id="rId1"/>
@@ -28,6 +28,17 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1655,6 +1666,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="43" fontId="40" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1694,18 +1714,9 @@
     <xf numFmtId="0" fontId="13" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Millares" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Normal 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
@@ -1732,9 +1743,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1772,7 +1783,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1878,7 +1889,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2020,7 +2031,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2033,28 +2044,28 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="42.85546875" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" customWidth="1"/>
-    <col min="5" max="5" width="20.5703125" style="102" customWidth="1"/>
-    <col min="6" max="6" width="23.28515625" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" customWidth="1"/>
-    <col min="8" max="8" width="20.85546875" customWidth="1"/>
-    <col min="9" max="9" width="19.140625" customWidth="1"/>
+    <col min="1" max="1" width="42.88671875" customWidth="1"/>
+    <col min="2" max="2" width="22.109375" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" customWidth="1"/>
+    <col min="4" max="4" width="23.5546875" customWidth="1"/>
+    <col min="5" max="5" width="20.5546875" style="102" customWidth="1"/>
+    <col min="6" max="6" width="23.33203125" customWidth="1"/>
+    <col min="7" max="7" width="21.6640625" customWidth="1"/>
+    <col min="8" max="8" width="20.88671875" customWidth="1"/>
+    <col min="9" max="9" width="19.109375" customWidth="1"/>
     <col min="10" max="10" width="20" style="102" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="20.28515625" style="102" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="20.7109375" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="24.42578125" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="24.28515625" customWidth="1"/>
-    <col min="15" max="15" width="2.28515625" customWidth="1"/>
-    <col min="16" max="16" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.33203125" style="102" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="20.6640625" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="24.44140625" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="24.33203125" customWidth="1"/>
+    <col min="15" max="15" width="2.33203125" customWidth="1"/>
+    <col min="16" max="16" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2066,26 +2077,26 @@
       <c r="I1" s="1"/>
       <c r="O1" s="14"/>
     </row>
-    <row r="2" spans="1:15" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="227" t="s">
+    <row r="2" spans="1:15" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="230" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="228"/>
-      <c r="C2" s="228"/>
-      <c r="D2" s="228"/>
-      <c r="E2" s="228"/>
-      <c r="F2" s="228"/>
-      <c r="G2" s="228"/>
-      <c r="H2" s="228"/>
-      <c r="I2" s="228"/>
-      <c r="J2" s="228"/>
-      <c r="K2" s="228"/>
-      <c r="L2" s="228"/>
-      <c r="M2" s="228"/>
-      <c r="N2" s="229"/>
+      <c r="B2" s="231"/>
+      <c r="C2" s="231"/>
+      <c r="D2" s="231"/>
+      <c r="E2" s="231"/>
+      <c r="F2" s="231"/>
+      <c r="G2" s="231"/>
+      <c r="H2" s="231"/>
+      <c r="I2" s="231"/>
+      <c r="J2" s="231"/>
+      <c r="K2" s="231"/>
+      <c r="L2" s="231"/>
+      <c r="M2" s="231"/>
+      <c r="N2" s="232"/>
       <c r="O2" s="14"/>
     </row>
-    <row r="3" spans="1:15" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
@@ -2097,69 +2108,69 @@
       <c r="I3" s="1"/>
       <c r="O3" s="14"/>
     </row>
-    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="230" t="s">
+    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="233" t="s">
         <v>93</v>
       </c>
-      <c r="B4" s="232" t="s">
+      <c r="B4" s="235" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="233" t="s">
+      <c r="C4" s="236" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="233" t="s">
+      <c r="D4" s="236" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="233" t="s">
+      <c r="E4" s="236" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="233" t="s">
+      <c r="F4" s="236" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="233" t="s">
+      <c r="G4" s="236" t="s">
         <v>68</v>
       </c>
-      <c r="H4" s="233" t="s">
+      <c r="H4" s="236" t="s">
         <v>69</v>
       </c>
-      <c r="I4" s="233" t="s">
+      <c r="I4" s="236" t="s">
         <v>38</v>
       </c>
-      <c r="J4" s="233" t="s">
+      <c r="J4" s="236" t="s">
         <v>39</v>
       </c>
-      <c r="K4" s="233" t="s">
+      <c r="K4" s="236" t="s">
         <v>60</v>
       </c>
-      <c r="L4" s="233" t="s">
+      <c r="L4" s="236" t="s">
         <v>42</v>
       </c>
-      <c r="M4" s="233" t="s">
+      <c r="M4" s="236" t="s">
         <v>63</v>
       </c>
-      <c r="N4" s="235" t="s">
+      <c r="N4" s="238" t="s">
         <v>7</v>
       </c>
       <c r="O4" s="14"/>
     </row>
-    <row r="5" spans="1:15" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="231"/>
-      <c r="B5" s="231"/>
-      <c r="C5" s="234"/>
-      <c r="D5" s="234"/>
-      <c r="E5" s="234"/>
-      <c r="F5" s="234"/>
-      <c r="G5" s="234"/>
-      <c r="H5" s="234"/>
-      <c r="I5" s="234"/>
-      <c r="J5" s="234"/>
-      <c r="K5" s="234"/>
-      <c r="L5" s="234"/>
-      <c r="M5" s="234"/>
-      <c r="N5" s="236"/>
+    <row r="5" spans="1:15" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="234"/>
+      <c r="B5" s="234"/>
+      <c r="C5" s="237"/>
+      <c r="D5" s="237"/>
+      <c r="E5" s="237"/>
+      <c r="F5" s="237"/>
+      <c r="G5" s="237"/>
+      <c r="H5" s="237"/>
+      <c r="I5" s="237"/>
+      <c r="J5" s="237"/>
+      <c r="K5" s="237"/>
+      <c r="L5" s="237"/>
+      <c r="M5" s="237"/>
+      <c r="N5" s="239"/>
       <c r="O5" s="14"/>
     </row>
-    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
         <v>21</v>
       </c>
@@ -2217,7 +2228,7 @@
       </c>
       <c r="O6" s="14"/>
     </row>
-    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>20</v>
       </c>
@@ -2275,7 +2286,7 @@
       </c>
       <c r="O7" s="14"/>
     </row>
-    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>41</v>
       </c>
@@ -2333,7 +2344,7 @@
       </c>
       <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>59</v>
       </c>
@@ -2391,7 +2402,7 @@
       </c>
       <c r="O9" s="14"/>
     </row>
-    <row r="10" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="66" t="s">
         <v>19</v>
       </c>
@@ -2449,7 +2460,7 @@
       </c>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="185" t="s">
         <v>6</v>
       </c>
@@ -2507,7 +2518,7 @@
       </c>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14"/>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
@@ -2524,7 +2535,7 @@
       <c r="N12" s="14"/>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="23" t="s">
         <v>58</v>
       </c>
@@ -2582,7 +2593,7 @@
       </c>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
@@ -2640,7 +2651,7 @@
       </c>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>90</v>
       </c>
@@ -2698,7 +2709,7 @@
       </c>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>84</v>
       </c>
@@ -2726,7 +2737,7 @@
       </c>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="1:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="44" t="s">
         <v>65</v>
       </c>
@@ -2784,7 +2795,7 @@
       </c>
       <c r="O17" s="14"/>
     </row>
-    <row r="18" spans="1:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="16" t="s">
         <v>16</v>
       </c>
@@ -2843,7 +2854,7 @@
       <c r="O18" s="14"/>
       <c r="P18" s="15"/>
     </row>
-    <row r="19" spans="1:17" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="45"/>
       <c r="B19" s="68"/>
       <c r="C19" s="68"/>
@@ -2862,7 +2873,7 @@
       <c r="P19" s="14"/>
       <c r="Q19" s="14"/>
     </row>
-    <row r="20" spans="1:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
         <v>4</v>
       </c>
@@ -2920,7 +2931,7 @@
       </c>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="10"/>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
@@ -2937,7 +2948,7 @@
       <c r="N21" s="11"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="82" t="s">
         <v>101</v>
       </c>
@@ -2956,7 +2967,7 @@
       <c r="N22" s="11"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="1:17" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="186" t="s">
         <v>54</v>
       </c>
@@ -2975,7 +2986,7 @@
       <c r="N23" s="195"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" spans="1:17" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:17" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="39"/>
       <c r="B24" s="112"/>
       <c r="C24" s="80"/>
@@ -2992,7 +3003,7 @@
       <c r="N24" s="195"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25" s="182" t="s">
         <v>71</v>
       </c>
@@ -3011,7 +3022,7 @@
       <c r="N25" s="14"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A26" s="151" t="s">
         <v>89</v>
       </c>
@@ -3030,7 +3041,7 @@
       <c r="N26" s="14"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A27" s="151" t="s">
         <v>76</v>
       </c>
@@ -3049,7 +3060,7 @@
       <c r="N27" s="14"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A28" s="151"/>
       <c r="B28" s="131"/>
       <c r="C28" s="80"/>
@@ -3066,7 +3077,7 @@
       <c r="N28" s="14"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A29" s="182" t="s">
         <v>70</v>
       </c>
@@ -3085,7 +3096,7 @@
       <c r="N29" s="14"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A30" s="151" t="s">
         <v>78</v>
       </c>
@@ -3104,7 +3115,7 @@
       <c r="N30" s="14"/>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A31" s="151" t="s">
         <v>77</v>
       </c>
@@ -3123,7 +3134,7 @@
       <c r="N31" s="14"/>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A32" s="151"/>
       <c r="B32" s="131"/>
       <c r="C32" s="80"/>
@@ -3140,7 +3151,7 @@
       <c r="N32" s="14"/>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="111" t="s">
         <v>35</v>
       </c>
@@ -3159,7 +3170,7 @@
       <c r="N33" s="14"/>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="111" t="s">
         <v>62</v>
       </c>
@@ -3178,7 +3189,7 @@
       <c r="N34" s="14"/>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="179"/>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
@@ -3194,16 +3205,16 @@
       <c r="M35" s="14"/>
       <c r="N35" s="14"/>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="H37" s="51"/>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="H38" s="51"/>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="H39" s="51"/>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="H40" s="51"/>
     </row>
   </sheetData>
@@ -3238,29 +3249,29 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:W35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="53.85546875" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="53.88671875" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" customWidth="1"/>
+    <col min="3" max="3" width="19.109375" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="18.28515625" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" customWidth="1"/>
     <col min="8" max="8" width="19" customWidth="1"/>
-    <col min="9" max="9" width="18.85546875" customWidth="1"/>
-    <col min="10" max="10" width="18.85546875" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="19.140625" style="102" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="18.88671875" customWidth="1"/>
+    <col min="10" max="10" width="18.88671875" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="19.109375" style="102" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="19" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="18.140625" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="19.42578125" customWidth="1"/>
-    <col min="15" max="15" width="19.5703125" customWidth="1"/>
-    <col min="16" max="16" width="13.28515625" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="11.42578125" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="1.85546875" customWidth="1"/>
+    <col min="13" max="13" width="18.109375" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="19.44140625" customWidth="1"/>
+    <col min="15" max="15" width="19.5546875" customWidth="1"/>
+    <col min="16" max="16" width="13.33203125" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="11.44140625" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="1.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3275,29 +3286,29 @@
       <c r="Q1" s="14"/>
       <c r="R1" s="14"/>
     </row>
-    <row r="2" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="237" t="s">
+    <row r="2" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="240" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="238"/>
-      <c r="C2" s="238"/>
-      <c r="D2" s="238"/>
-      <c r="E2" s="238"/>
-      <c r="F2" s="238"/>
-      <c r="G2" s="238"/>
-      <c r="H2" s="238"/>
-      <c r="I2" s="238"/>
-      <c r="J2" s="238"/>
-      <c r="K2" s="238"/>
-      <c r="L2" s="238"/>
-      <c r="M2" s="238"/>
-      <c r="N2" s="239"/>
+      <c r="B2" s="241"/>
+      <c r="C2" s="241"/>
+      <c r="D2" s="241"/>
+      <c r="E2" s="241"/>
+      <c r="F2" s="241"/>
+      <c r="G2" s="241"/>
+      <c r="H2" s="241"/>
+      <c r="I2" s="241"/>
+      <c r="J2" s="241"/>
+      <c r="K2" s="241"/>
+      <c r="L2" s="241"/>
+      <c r="M2" s="241"/>
+      <c r="N2" s="242"/>
       <c r="O2" s="14"/>
       <c r="P2" s="14"/>
       <c r="Q2" s="14"/>
       <c r="R2" s="14"/>
     </row>
-    <row r="3" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
@@ -3312,7 +3323,7 @@
       <c r="Q3" s="14"/>
       <c r="R3" s="14"/>
     </row>
-    <row r="4" spans="1:23" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
@@ -3360,7 +3371,7 @@
       <c r="Q4" s="14"/>
       <c r="R4" s="14"/>
     </row>
-    <row r="5" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="105" t="s">
         <v>5</v>
       </c>
@@ -3399,7 +3410,7 @@
       <c r="Q5" s="14"/>
       <c r="R5" s="14"/>
     </row>
-    <row r="6" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="106" t="s">
         <v>52</v>
       </c>
@@ -3424,7 +3435,7 @@
       <c r="Q6" s="14"/>
       <c r="R6" s="14"/>
     </row>
-    <row r="7" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="107" t="s">
         <v>45</v>
       </c>
@@ -3463,7 +3474,7 @@
       <c r="Q7" s="14"/>
       <c r="R7" s="14"/>
     </row>
-    <row r="8" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="107" t="s">
         <v>10</v>
       </c>
@@ -3488,7 +3499,7 @@
       <c r="Q8" s="14"/>
       <c r="R8" s="14"/>
     </row>
-    <row r="9" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="107" t="s">
         <v>50</v>
       </c>
@@ -3513,7 +3524,7 @@
       <c r="Q9" s="14"/>
       <c r="R9" s="14"/>
     </row>
-    <row r="10" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="108" t="s">
         <v>37</v>
       </c>
@@ -3552,7 +3563,7 @@
       <c r="Q10" s="14"/>
       <c r="R10" s="14"/>
     </row>
-    <row r="11" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="109" t="s">
         <v>11</v>
       </c>
@@ -3577,7 +3588,7 @@
       <c r="Q11" s="14"/>
       <c r="R11" s="14"/>
     </row>
-    <row r="12" spans="1:23" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="16" t="s">
         <v>6</v>
       </c>
@@ -3638,7 +3649,7 @@
       <c r="Q12" s="14"/>
       <c r="R12" s="14"/>
     </row>
-    <row r="13" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>24</v>
       </c>
@@ -3681,7 +3692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="46" t="s">
         <v>25</v>
       </c>
@@ -3720,7 +3731,7 @@
       <c r="Q14" s="14"/>
       <c r="R14" s="14"/>
     </row>
-    <row r="15" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>51</v>
       </c>
@@ -3745,7 +3756,7 @@
       <c r="Q15" s="14"/>
       <c r="R15" s="14"/>
     </row>
-    <row r="16" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="16" t="s">
         <v>16</v>
       </c>
@@ -3806,7 +3817,7 @@
       <c r="Q16" s="14"/>
       <c r="R16" s="14"/>
     </row>
-    <row r="17" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3"/>
       <c r="B17" s="61"/>
       <c r="C17" s="61"/>
@@ -3830,7 +3841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
         <v>4</v>
       </c>
@@ -3891,7 +3902,7 @@
       <c r="Q18" s="14"/>
       <c r="R18" s="14"/>
     </row>
-    <row r="19" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="10"/>
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
@@ -3911,7 +3922,7 @@
       <c r="Q19" s="14"/>
       <c r="R19" s="14"/>
     </row>
-    <row r="20" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="82" t="s">
         <v>101</v>
       </c>
@@ -3935,7 +3946,7 @@
       <c r="S20" s="14"/>
       <c r="T20" s="14"/>
     </row>
-    <row r="21" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="82" t="s">
         <v>22</v>
       </c>
@@ -3959,7 +3970,7 @@
       <c r="S21" s="14"/>
       <c r="T21" s="14"/>
     </row>
-    <row r="22" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="179" t="s">
         <v>57</v>
       </c>
@@ -3983,7 +3994,7 @@
       <c r="S22" s="14"/>
       <c r="T22" s="14"/>
     </row>
-    <row r="23" spans="1:23" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" ht="10.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="178"/>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
@@ -4005,7 +4016,7 @@
       <c r="S23" s="14"/>
       <c r="T23" s="14"/>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" s="113" t="s">
         <v>26</v>
       </c>
@@ -4029,7 +4040,7 @@
       <c r="S24" s="14"/>
       <c r="T24" s="14"/>
     </row>
-    <row r="25" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="151" t="s">
         <v>74</v>
       </c>
@@ -4053,7 +4064,7 @@
       <c r="S25" s="14"/>
       <c r="T25" s="14"/>
     </row>
-    <row r="26" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="151" t="s">
         <v>75</v>
       </c>
@@ -4077,7 +4088,7 @@
       <c r="S26" s="14"/>
       <c r="T26" s="14"/>
     </row>
-    <row r="27" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="151"/>
       <c r="B27" s="114"/>
       <c r="C27" s="114"/>
@@ -4099,7 +4110,7 @@
       <c r="S27" s="14"/>
       <c r="T27" s="14"/>
     </row>
-    <row r="28" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="111" t="s">
         <v>34</v>
       </c>
@@ -4123,7 +4134,7 @@
       <c r="S28" s="14"/>
       <c r="T28" s="14"/>
     </row>
-    <row r="29" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="111" t="s">
         <v>61</v>
       </c>
@@ -4147,7 +4158,7 @@
       <c r="S29" s="14"/>
       <c r="T29" s="14"/>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" s="111"/>
       <c r="B30" s="14"/>
       <c r="C30" s="14"/>
@@ -4169,7 +4180,7 @@
       <c r="S30" s="14"/>
       <c r="T30" s="14"/>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" s="14"/>
       <c r="B31" s="14"/>
       <c r="C31" s="14"/>
@@ -4191,7 +4202,7 @@
       <c r="S31" s="14"/>
       <c r="T31" s="14"/>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
@@ -4213,7 +4224,7 @@
       <c r="S32" s="14"/>
       <c r="T32" s="14"/>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" s="14"/>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -4235,7 +4246,7 @@
       <c r="S33" s="14"/>
       <c r="T33" s="14"/>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" s="14"/>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
@@ -4257,7 +4268,7 @@
       <c r="S34" s="14"/>
       <c r="T34" s="14"/>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35" s="14"/>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
@@ -4296,27 +4307,27 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="49.85546875" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" customWidth="1"/>
-    <col min="5" max="5" width="21.28515625" customWidth="1"/>
-    <col min="6" max="6" width="20.42578125" customWidth="1"/>
-    <col min="7" max="7" width="18.28515625" customWidth="1"/>
-    <col min="8" max="8" width="18.28515625" style="102" customWidth="1"/>
-    <col min="9" max="9" width="18.42578125" customWidth="1"/>
-    <col min="10" max="10" width="0.140625" style="102" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="19.85546875" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="20.85546875" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="19.28515625" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="19.28515625" customWidth="1"/>
-    <col min="15" max="15" width="6.5703125" customWidth="1"/>
+    <col min="1" max="1" width="49.88671875" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" customWidth="1"/>
+    <col min="5" max="5" width="21.33203125" customWidth="1"/>
+    <col min="6" max="6" width="20.44140625" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" customWidth="1"/>
+    <col min="8" max="8" width="18.33203125" style="102" customWidth="1"/>
+    <col min="9" max="9" width="18.44140625" customWidth="1"/>
+    <col min="10" max="10" width="0.109375" style="102" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="19.88671875" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="20.88671875" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="19.33203125" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="19.33203125" customWidth="1"/>
+    <col min="15" max="15" width="6.5546875" customWidth="1"/>
     <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="29"/>
       <c r="B1" s="29"/>
       <c r="C1" s="29"/>
@@ -4332,26 +4343,26 @@
       <c r="M1" s="14"/>
       <c r="N1" s="14"/>
     </row>
-    <row r="2" spans="1:18" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="240" t="s">
+    <row r="2" spans="1:18" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="227" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="241"/>
-      <c r="C2" s="241"/>
-      <c r="D2" s="241"/>
-      <c r="E2" s="241"/>
-      <c r="F2" s="241"/>
-      <c r="G2" s="241"/>
-      <c r="H2" s="241"/>
-      <c r="I2" s="241"/>
-      <c r="J2" s="241"/>
-      <c r="K2" s="241"/>
-      <c r="L2" s="241"/>
-      <c r="M2" s="241"/>
-      <c r="N2" s="242"/>
+      <c r="B2" s="228"/>
+      <c r="C2" s="228"/>
+      <c r="D2" s="228"/>
+      <c r="E2" s="228"/>
+      <c r="F2" s="228"/>
+      <c r="G2" s="228"/>
+      <c r="H2" s="228"/>
+      <c r="I2" s="228"/>
+      <c r="J2" s="228"/>
+      <c r="K2" s="228"/>
+      <c r="L2" s="228"/>
+      <c r="M2" s="228"/>
+      <c r="N2" s="229"/>
       <c r="O2" s="14"/>
     </row>
-    <row r="3" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="29"/>
       <c r="B3" s="29"/>
       <c r="C3" s="30"/>
@@ -4366,7 +4377,7 @@
       <c r="N3" s="14"/>
       <c r="O3" s="14"/>
     </row>
-    <row r="4" spans="1:18" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="31" t="s">
         <v>8</v>
       </c>
@@ -4412,7 +4423,7 @@
       <c r="O4" s="14"/>
       <c r="Q4" s="43"/>
     </row>
-    <row r="5" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>55</v>
       </c>
@@ -4448,7 +4459,7 @@
       </c>
       <c r="O5" s="62"/>
     </row>
-    <row r="6" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="70" t="s">
         <v>79</v>
       </c>
@@ -4486,7 +4497,7 @@
       <c r="O6" s="134"/>
       <c r="P6" s="206"/>
     </row>
-    <row r="7" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
@@ -4509,7 +4520,7 @@
       <c r="O7" s="14"/>
       <c r="P7" s="42"/>
     </row>
-    <row r="8" spans="1:18" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="70" t="s">
         <v>81</v>
       </c>
@@ -4547,7 +4558,7 @@
       <c r="O8" s="14"/>
       <c r="P8" s="206"/>
     </row>
-    <row r="9" spans="1:18" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="171" t="s">
         <v>82</v>
       </c>
@@ -4571,7 +4582,7 @@
       <c r="P9" s="51"/>
       <c r="R9" s="210"/>
     </row>
-    <row r="10" spans="1:18" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="89" t="s">
         <v>91</v>
       </c>
@@ -4629,7 +4640,7 @@
       </c>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="1:18" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="22"/>
       <c r="B11" s="76"/>
       <c r="C11" s="76"/>
@@ -4649,7 +4660,7 @@
       </c>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="1:18" ht="18.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="18.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="89" t="s">
         <v>15</v>
       </c>
@@ -4707,7 +4718,7 @@
       </c>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="1:18" s="14" customFormat="1" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" s="14" customFormat="1" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="148">
         <v>0</v>
       </c>
@@ -4728,7 +4739,7 @@
       <c r="M13" s="141"/>
       <c r="N13" s="62"/>
     </row>
-    <row r="14" spans="1:18" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="16" t="s">
         <v>6</v>
       </c>
@@ -4786,7 +4797,7 @@
       </c>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14"/>
       <c r="B15" s="148"/>
       <c r="C15" s="148"/>
@@ -4803,7 +4814,7 @@
       <c r="N15" s="62"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="23" t="s">
         <v>53</v>
       </c>
@@ -4839,7 +4850,7 @@
       </c>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="1:18" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>23</v>
       </c>
@@ -4878,7 +4889,7 @@
       <c r="P17" s="51"/>
       <c r="Q17" s="51"/>
     </row>
-    <row r="18" spans="1:18" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="70" t="s">
         <v>46</v>
       </c>
@@ -4900,7 +4911,7 @@
       </c>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="1:18" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="220" t="s">
         <v>73</v>
       </c>
@@ -4924,7 +4935,7 @@
       </c>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="1:18" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="225" t="s">
         <v>16</v>
       </c>
@@ -4982,7 +4993,7 @@
       </c>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="1:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="27"/>
       <c r="B21" s="136"/>
       <c r="C21" s="136"/>
@@ -4999,7 +5010,7 @@
       <c r="N21" s="224"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="1:18" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="212"/>
       <c r="B22" s="26"/>
       <c r="C22" s="26"/>
@@ -5022,7 +5033,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="70"/>
       <c r="B23" s="19">
         <v>0</v>
@@ -5074,7 +5085,7 @@
         <v>418900</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="19.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" ht="19.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="183"/>
       <c r="B24" s="28">
         <f t="shared" ref="B24:M24" si="6">+SUM(B22:B23)</f>
@@ -5131,7 +5142,7 @@
       <c r="O24" s="14"/>
       <c r="Q24" s="94"/>
     </row>
-    <row r="25" spans="1:18" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="136"/>
       <c r="C25" s="136"/>
       <c r="D25" s="136"/>
@@ -5147,7 +5158,7 @@
       <c r="N25" s="42"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="1:18" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="16" t="s">
         <v>16</v>
       </c>
@@ -5206,7 +5217,7 @@
       <c r="O26" s="14"/>
       <c r="Q26" s="51"/>
     </row>
-    <row r="27" spans="1:18" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="136"/>
       <c r="C27" s="136"/>
       <c r="D27" s="136"/>
@@ -5224,7 +5235,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="184" t="s">
         <v>17</v>
       </c>
@@ -5282,7 +5293,7 @@
       </c>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="111"/>
       <c r="B29" s="29"/>
       <c r="C29" s="29"/>
@@ -5299,7 +5310,7 @@
       <c r="N29" s="14"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" s="82" t="s">
         <v>101</v>
       </c>
@@ -5318,7 +5329,7 @@
       <c r="N30" s="80"/>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="82" t="s">
         <v>22</v>
       </c>
@@ -5340,7 +5351,7 @@
       <c r="N31" s="131"/>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="179" t="s">
         <v>57</v>
       </c>
@@ -5359,7 +5370,7 @@
       <c r="N32" s="131"/>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="177"/>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -5376,7 +5387,7 @@
       <c r="N33" s="131"/>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="113" t="s">
         <v>26</v>
       </c>
@@ -5395,7 +5406,7 @@
       <c r="N34" s="14"/>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="151" t="s">
         <v>87</v>
       </c>
@@ -5414,7 +5425,7 @@
       <c r="N35" s="14"/>
       <c r="O35" s="14"/>
     </row>
-    <row r="36" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="151" t="s">
         <v>88</v>
       </c>
@@ -5433,7 +5444,7 @@
       <c r="N36" s="14"/>
       <c r="O36" s="14"/>
     </row>
-    <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="151"/>
       <c r="B37" s="114"/>
       <c r="C37" s="114"/>
@@ -5450,7 +5461,7 @@
       <c r="N37" s="14"/>
       <c r="O37" s="14"/>
     </row>
-    <row r="38" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="111" t="s">
         <v>34</v>
       </c>
@@ -5469,7 +5480,7 @@
       <c r="N38" s="14"/>
       <c r="O38" s="14"/>
     </row>
-    <row r="39" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="111" t="s">
         <v>61</v>
       </c>
@@ -5488,7 +5499,7 @@
       <c r="N39" s="14"/>
       <c r="O39" s="14"/>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="111"/>
       <c r="B40" s="14"/>
       <c r="C40" s="14"/>
@@ -5504,13 +5515,13 @@
       <c r="M40" s="40"/>
       <c r="N40" s="40"/>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="39"/>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="39"/>
     </row>
-    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="B43" s="41">
         <v>34000</v>
       </c>
@@ -5518,7 +5529,7 @@
         <v>44000</v>
       </c>
     </row>
-    <row r="44" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" s="41">
         <v>66111</v>
       </c>
@@ -5526,7 +5537,7 @@
         <v>76305</v>
       </c>
     </row>
-    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" s="42">
         <f>SUM(B43:B44)</f>
         <v>100111</v>
@@ -5536,12 +5547,12 @@
         <v>120305</v>
       </c>
     </row>
-    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="F46" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="47" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>28</v>
       </c>
@@ -5560,7 +5571,7 @@
         <v>323383.18064516131</v>
       </c>
     </row>
-    <row r="48" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="43" t="s">
         <v>27</v>
       </c>
@@ -5576,10 +5587,10 @@
         <v>31</v>
       </c>
     </row>
-    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="39"/>
     </row>
-    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>29</v>
       </c>
@@ -5591,7 +5602,7 @@
         <v>44576.9375</v>
       </c>
     </row>
-    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="43" t="s">
         <v>30</v>
       </c>
@@ -5607,23 +5618,23 @@
         <v>31</v>
       </c>
     </row>
-    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="B52" s="42"/>
       <c r="C52" s="91"/>
       <c r="D52" s="92"/>
     </row>
-    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="B53" s="42"/>
       <c r="C53" s="91"/>
       <c r="D53" s="92"/>
     </row>
-    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="B54" s="42"/>
       <c r="C54" s="91"/>
       <c r="D54" s="92"/>
     </row>
-    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>32</v>
       </c>
@@ -5631,7 +5642,7 @@
         <v>44607.9375</v>
       </c>
     </row>
-    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>33</v>
       </c>
@@ -5643,10 +5654,10 @@
         <v>28</v>
       </c>
     </row>
-    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="123">
         <v>120</v>
       </c>
@@ -5677,26 +5688,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="A1:R61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="53.42578125" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" hidden="1" customWidth="1"/>
-    <col min="3" max="4" width="18.28515625" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="17.7109375" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="20.42578125" customWidth="1"/>
-    <col min="7" max="7" width="18.28515625" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" style="102" customWidth="1"/>
+    <col min="1" max="1" width="53.44140625" customWidth="1"/>
+    <col min="2" max="2" width="24.5546875" hidden="1" customWidth="1"/>
+    <col min="3" max="4" width="18.33203125" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="20.44140625" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" customWidth="1"/>
+    <col min="8" max="8" width="16.33203125" style="102" customWidth="1"/>
     <col min="9" max="9" width="19" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="0.140625" style="102" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="19.85546875" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="20.85546875" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="19.28515625" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="19.28515625" customWidth="1"/>
-    <col min="15" max="15" width="6.5703125" customWidth="1"/>
+    <col min="10" max="10" width="0.109375" style="102" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="19.88671875" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="20.88671875" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="19.33203125" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="19.33203125" customWidth="1"/>
+    <col min="15" max="15" width="6.5546875" customWidth="1"/>
     <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="29"/>
       <c r="B1" s="29"/>
       <c r="C1" s="29"/>
@@ -5712,26 +5723,26 @@
       <c r="M1" s="14"/>
       <c r="N1" s="14"/>
     </row>
-    <row r="2" spans="1:18" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="240" t="s">
+    <row r="2" spans="1:18" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="227" t="s">
         <v>92</v>
       </c>
-      <c r="B2" s="241"/>
-      <c r="C2" s="241"/>
-      <c r="D2" s="241"/>
-      <c r="E2" s="241"/>
-      <c r="F2" s="241"/>
-      <c r="G2" s="241"/>
-      <c r="H2" s="241"/>
-      <c r="I2" s="241"/>
-      <c r="J2" s="241"/>
-      <c r="K2" s="241"/>
-      <c r="L2" s="241"/>
-      <c r="M2" s="241"/>
-      <c r="N2" s="242"/>
+      <c r="B2" s="228"/>
+      <c r="C2" s="228"/>
+      <c r="D2" s="228"/>
+      <c r="E2" s="228"/>
+      <c r="F2" s="228"/>
+      <c r="G2" s="228"/>
+      <c r="H2" s="228"/>
+      <c r="I2" s="228"/>
+      <c r="J2" s="228"/>
+      <c r="K2" s="228"/>
+      <c r="L2" s="228"/>
+      <c r="M2" s="228"/>
+      <c r="N2" s="229"/>
       <c r="O2" s="14"/>
     </row>
-    <row r="3" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="29"/>
       <c r="B3" s="29"/>
       <c r="C3" s="30"/>
@@ -5746,7 +5757,7 @@
       <c r="N3" s="14"/>
       <c r="O3" s="14"/>
     </row>
-    <row r="4" spans="1:18" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="31" t="s">
         <v>8</v>
       </c>
@@ -5788,7 +5799,7 @@
       <c r="O4" s="14"/>
       <c r="Q4" s="43"/>
     </row>
-    <row r="5" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>96</v>
       </c>
@@ -5814,7 +5825,7 @@
       </c>
       <c r="O5" s="62"/>
     </row>
-    <row r="6" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="70" t="s">
         <v>97</v>
       </c>
@@ -5837,7 +5848,7 @@
       <c r="O6" s="134"/>
       <c r="P6" s="206"/>
     </row>
-    <row r="7" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
@@ -5860,7 +5871,7 @@
       <c r="O7" s="14"/>
       <c r="P7" s="42"/>
     </row>
-    <row r="8" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="70" t="s">
         <v>98</v>
       </c>
@@ -5885,7 +5896,7 @@
       <c r="O8" s="14"/>
       <c r="P8" s="206"/>
     </row>
-    <row r="9" spans="1:18" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="171" t="s">
         <v>82</v>
       </c>
@@ -5906,7 +5917,7 @@
       <c r="P9" s="51"/>
       <c r="R9" s="210"/>
     </row>
-    <row r="10" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="89" t="s">
         <v>13</v>
       </c>
@@ -5949,7 +5960,7 @@
       </c>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="1:18" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="22" t="s">
         <v>14</v>
       </c>
@@ -5971,7 +5982,7 @@
       </c>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="1:18" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="89" t="s">
         <v>15</v>
       </c>
@@ -6014,7 +6025,7 @@
       </c>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="1:18" s="14" customFormat="1" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" s="14" customFormat="1" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="148"/>
       <c r="C13" s="148"/>
       <c r="D13" s="148"/>
@@ -6029,7 +6040,7 @@
       <c r="M13" s="141"/>
       <c r="N13" s="62"/>
     </row>
-    <row r="14" spans="1:18" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="16" t="s">
         <v>6</v>
       </c>
@@ -6072,7 +6083,7 @@
       </c>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14"/>
       <c r="B15" s="148"/>
       <c r="C15" s="148"/>
@@ -6089,7 +6100,7 @@
       <c r="N15" s="62"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="23" t="s">
         <v>83</v>
       </c>
@@ -6111,7 +6122,7 @@
       </c>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>99</v>
       </c>
@@ -6137,7 +6148,7 @@
       <c r="P17" s="51"/>
       <c r="Q17" s="51"/>
     </row>
-    <row r="18" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="70" t="s">
         <v>100</v>
       </c>
@@ -6163,7 +6174,7 @@
       </c>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="220" t="s">
         <v>73</v>
       </c>
@@ -6185,7 +6196,7 @@
       </c>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="222" t="s">
         <v>16</v>
       </c>
@@ -6228,7 +6239,7 @@
       </c>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="1:18" ht="0.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" ht="0.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="27"/>
       <c r="B21" s="136"/>
       <c r="C21" s="136"/>
@@ -6245,7 +6256,7 @@
       <c r="N21" s="63"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="1:18" ht="0.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" ht="0.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="209" t="s">
         <v>66</v>
       </c>
@@ -6269,7 +6280,7 @@
       </c>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="1:18" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="207" t="s">
         <v>64</v>
       </c>
@@ -6306,7 +6317,7 @@
       <c r="O23" s="62"/>
       <c r="R23" s="210"/>
     </row>
-    <row r="24" spans="1:18" ht="19.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" ht="19.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="183" t="s">
         <v>56</v>
       </c>
@@ -6350,7 +6361,7 @@
       <c r="O24" s="14"/>
       <c r="Q24" s="94"/>
     </row>
-    <row r="25" spans="1:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="136"/>
       <c r="C25" s="136"/>
       <c r="D25" s="136"/>
@@ -6366,7 +6377,7 @@
       <c r="N25" s="42"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="1:18" ht="21" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" ht="21" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="16" t="s">
         <v>16</v>
       </c>
@@ -6410,7 +6421,7 @@
       <c r="O26" s="14"/>
       <c r="Q26" s="51"/>
     </row>
-    <row r="27" spans="1:18" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="136"/>
       <c r="C27" s="136"/>
       <c r="D27" s="136"/>
@@ -6428,7 +6439,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="184" t="s">
         <v>17</v>
       </c>
@@ -6471,7 +6482,7 @@
       </c>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="111"/>
       <c r="B29" s="29"/>
       <c r="C29" s="29"/>
@@ -6488,7 +6499,7 @@
       <c r="N29" s="14"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" s="82" t="s">
         <v>101</v>
       </c>
@@ -6507,7 +6518,7 @@
       <c r="N30" s="80"/>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="82" t="s">
         <v>22</v>
       </c>
@@ -6529,7 +6540,7 @@
       <c r="N31" s="131"/>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="179"/>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
@@ -6546,7 +6557,7 @@
       <c r="N32" s="131"/>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="177"/>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -6563,7 +6574,7 @@
       <c r="N33" s="131"/>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="113" t="s">
         <v>26</v>
       </c>
@@ -6582,7 +6593,7 @@
       <c r="N34" s="14"/>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="151" t="s">
         <v>94</v>
       </c>
@@ -6601,7 +6612,7 @@
       <c r="N35" s="14"/>
       <c r="O35" s="14"/>
     </row>
-    <row r="36" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="151" t="s">
         <v>95</v>
       </c>
@@ -6620,7 +6631,7 @@
       <c r="N36" s="14"/>
       <c r="O36" s="14"/>
     </row>
-    <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="151"/>
       <c r="B37" s="114"/>
       <c r="C37" s="114"/>
@@ -6637,7 +6648,7 @@
       <c r="N37" s="14"/>
       <c r="O37" s="14"/>
     </row>
-    <row r="38" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="111"/>
       <c r="B38" s="114"/>
       <c r="C38" s="114"/>
@@ -6654,7 +6665,7 @@
       <c r="N38" s="14"/>
       <c r="O38" s="14"/>
     </row>
-    <row r="39" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="111"/>
       <c r="B39" s="114"/>
       <c r="C39" s="114"/>
@@ -6671,7 +6682,7 @@
       <c r="N39" s="14"/>
       <c r="O39" s="14"/>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="111"/>
       <c r="B40" s="14"/>
       <c r="C40" s="14"/>
@@ -6687,13 +6698,13 @@
       <c r="M40" s="40"/>
       <c r="N40" s="40"/>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="39"/>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="39"/>
     </row>
-    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="B43" s="41">
         <v>34000</v>
       </c>
@@ -6701,7 +6712,7 @@
         <v>44000</v>
       </c>
     </row>
-    <row r="44" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" s="41">
         <v>66111</v>
       </c>
@@ -6709,7 +6720,7 @@
         <v>76305</v>
       </c>
     </row>
-    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" s="42">
         <f>SUM(B43:B44)</f>
         <v>100111</v>
@@ -6719,12 +6730,12 @@
         <v>120305</v>
       </c>
     </row>
-    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="F46" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="47" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>28</v>
       </c>
@@ -6743,7 +6754,7 @@
         <v>323383.18064516131</v>
       </c>
     </row>
-    <row r="48" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="43" t="s">
         <v>27</v>
       </c>
@@ -6759,10 +6770,10 @@
         <v>31</v>
       </c>
     </row>
-    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="39"/>
     </row>
-    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>29</v>
       </c>
@@ -6774,7 +6785,7 @@
         <v>44576.9375</v>
       </c>
     </row>
-    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="43" t="s">
         <v>30</v>
       </c>
@@ -6790,23 +6801,23 @@
         <v>31</v>
       </c>
     </row>
-    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="B52" s="42"/>
       <c r="C52" s="91"/>
       <c r="D52" s="92"/>
     </row>
-    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="B53" s="42"/>
       <c r="C53" s="91"/>
       <c r="D53" s="92"/>
     </row>
-    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="B54" s="42"/>
       <c r="C54" s="91"/>
       <c r="D54" s="92"/>
     </row>
-    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>32</v>
       </c>
@@ -6814,7 +6825,7 @@
         <v>44607.9375</v>
       </c>
     </row>
-    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>33</v>
       </c>
@@ -6826,10 +6837,10 @@
         <v>28</v>
       </c>
     </row>
-    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="123">
         <v>120</v>
       </c>

</xml_diff>